<commit_message>
Publish validated Full Online Archive Edition
</commit_message>
<xml_diff>
--- a/full/exports/Welsh-LDS-Branches-Canonical-and-Possible.xlsx
+++ b/full/exports/Welsh-LDS-Branches-Canonical-and-Possible.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical" sheetId="1" r:id="R546cca3ce3524535"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Possible" sheetId="2" r:id="R2804320de7e74f0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical" sheetId="1" r:id="Rff8079f200ec4edb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Possible" sheetId="2" r:id="R8e42c2db7a05488a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2313,7 +2313,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60d3e5dd1d0449ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a7ceba41bae47c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2841,7 +2841,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6aa30af83662447e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R109afa6e11d7476e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish current Full Online Archive Edition
</commit_message>
<xml_diff>
--- a/full/exports/Welsh-LDS-Branches-Canonical-and-Possible.xlsx
+++ b/full/exports/Welsh-LDS-Branches-Canonical-and-Possible.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical" sheetId="1" r:id="Rff8079f200ec4edb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Possible" sheetId="2" r:id="R8e42c2db7a05488a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical" sheetId="1" r:id="R18742ee2750447ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Possible" sheetId="2" r:id="Rd217860ab4374f4a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2313,7 +2313,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a7ceba41bae47c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24101063ab4b4461"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2841,7 +2841,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R109afa6e11d7476e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf98636e08be94ba4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish publication viewer and catalog polish
</commit_message>
<xml_diff>
--- a/full/exports/Welsh-LDS-Branches-Canonical-and-Possible.xlsx
+++ b/full/exports/Welsh-LDS-Branches-Canonical-and-Possible.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical" sheetId="1" r:id="R18742ee2750447ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Possible" sheetId="2" r:id="Rd217860ab4374f4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical" sheetId="1" r:id="Raebf3ec6802342eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Possible" sheetId="2" r:id="R455446f39fde4b4f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2313,7 +2313,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24101063ab4b4461"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e51ed9e964044e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2841,7 +2841,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf98636e08be94ba4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb18c429ae65f4fae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish validated archive interface updates
</commit_message>
<xml_diff>
--- a/full/exports/Welsh-LDS-Branches-Canonical-and-Possible.xlsx
+++ b/full/exports/Welsh-LDS-Branches-Canonical-and-Possible.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical" sheetId="1" r:id="Raebf3ec6802342eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Possible" sheetId="2" r:id="R455446f39fde4b4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical" sheetId="1" r:id="Rc10b6efd40bc4466"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Possible" sheetId="2" r:id="R44fee4ed9f694a23"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2313,7 +2313,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e51ed9e964044e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6d8f7f747654fd0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2510,7 +2510,7 @@
       <x:c r="C11" s="6" t="str"/>
       <x:c r="D11" s="6" t="str"/>
       <x:c r="E11" s="5" t="str">
-        <x:v>Historical branch-like reference; locality unresolved.</x:v>
+        <x:v>Probable source variant of Cog/Cogan; exact cause of the spelling difference unresolved.</x:v>
       </x:c>
       <x:c r="F11" s="5" t="str"/>
       <x:c r="G11" s="5" t="str"/>
@@ -2841,7 +2841,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb18c429ae65f4fae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2bf0df57b764e9d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish validated archive search and viewer updates
</commit_message>
<xml_diff>
--- a/full/exports/Welsh-LDS-Branches-Canonical-and-Possible.xlsx
+++ b/full/exports/Welsh-LDS-Branches-Canonical-and-Possible.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical" sheetId="1" r:id="Rc10b6efd40bc4466"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Possible" sheetId="2" r:id="R44fee4ed9f694a23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical" sheetId="1" r:id="R97d1452e54ea4157"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Possible" sheetId="2" r:id="R6d17f3226c684b7a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2313,7 +2313,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6d8f7f747654fd0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02e54abdc6e5426c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2841,7 +2841,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2bf0df57b764e9d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3b776645baf40c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Promote validated review state to full archive
</commit_message>
<xml_diff>
--- a/full/exports/Welsh-LDS-Branches-Canonical-and-Possible.xlsx
+++ b/full/exports/Welsh-LDS-Branches-Canonical-and-Possible.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical" sheetId="1" r:id="R97d1452e54ea4157"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Possible" sheetId="2" r:id="R6d17f3226c684b7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical" sheetId="1" r:id="R2867df89e0684d5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Possible" sheetId="2" r:id="R841b0fada9274cd0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2313,7 +2313,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02e54abdc6e5426c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45f24b876eb14d32"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2841,7 +2841,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3b776645baf40c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R204719ebd797405d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>